<commit_message>
qa: record round 5 black-box test results (live NVIDIA assistant)
Round 5 ran against the real backend with a live NVIDIA model instead
of the mock, seeded a fresh account with AI consent pre-granted. Nine
issues found (1 blocker: broken shelf add-books dialog; 3 major: lost
session reflection, off-topic assistant timeouts, unexplained logout;
rest minor/polish). No fixes applied yet -- recording results only.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/qa/blackbox-test-log.xlsx
+++ b/docs/qa/blackbox-test-log.xlsx
@@ -13,9 +13,10 @@
     <sheet name="Round 2" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="Round 3" sheetId="5" state="visible" r:id="rId5"/>
     <sheet name="Round 4" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Round 5" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'All issues'!$A$1:$N$79</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'All issues'!$A$1:$N$88</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -491,7 +492,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E23"/>
+  <dimension ref="A1:F24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -499,6 +500,7 @@
     <col width="11" customWidth="1" min="3" max="3"/>
     <col width="11" customWidth="1" min="4" max="4"/>
     <col width="11" customWidth="1" min="5" max="5"/>
+    <col width="11" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -534,6 +536,11 @@
           <t>Round 4</t>
         </is>
       </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>Round 5</t>
+        </is>
+      </c>
     </row>
     <row r="4"/>
     <row r="5">
@@ -554,6 +561,9 @@
       <c r="E5" s="4" t="n">
         <v>7</v>
       </c>
+      <c r="F5" s="5" t="n">
+        <v>8</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
@@ -573,6 +583,9 @@
       <c r="E6" s="4" t="n">
         <v>6</v>
       </c>
+      <c r="F6" s="4" t="n">
+        <v>7</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
@@ -592,6 +605,9 @@
       <c r="E7" s="4" t="n">
         <v>6</v>
       </c>
+      <c r="F7" s="5" t="n">
+        <v>8</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
@@ -613,6 +629,9 @@
       <c r="E8" s="4" t="n">
         <v>5</v>
       </c>
+      <c r="F8" s="5" t="n">
+        <v>9</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
@@ -632,6 +651,9 @@
       <c r="E9" s="5" t="n">
         <v>8</v>
       </c>
+      <c r="F9" s="4" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
@@ -651,6 +673,9 @@
       <c r="E10" s="5" t="n">
         <v>8</v>
       </c>
+      <c r="F10" s="4" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
@@ -670,6 +695,9 @@
       <c r="E11" s="4" t="n">
         <v>5</v>
       </c>
+      <c r="F11" s="4" t="n">
+        <v>7</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
@@ -689,6 +717,9 @@
       <c r="E12" s="4" t="n">
         <v>7</v>
       </c>
+      <c r="F12" s="4" t="n">
+        <v>7</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
@@ -708,6 +739,9 @@
       <c r="E13" s="5" t="n">
         <v>8</v>
       </c>
+      <c r="F13" s="5" t="n">
+        <v>9</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
@@ -727,6 +761,9 @@
       <c r="E14" s="4" t="n">
         <v>6</v>
       </c>
+      <c r="F14" s="4" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
@@ -746,6 +783,9 @@
       <c r="E15" s="4" t="n">
         <v>6</v>
       </c>
+      <c r="F15" s="4" t="n">
+        <v>7</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="7" t="inlineStr">
@@ -765,6 +805,9 @@
       <c r="E16" s="3" t="n">
         <v>5</v>
       </c>
+      <c r="F16" s="3" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="7" t="inlineStr">
@@ -784,6 +827,9 @@
       <c r="E17" s="3" t="n">
         <v>17</v>
       </c>
+      <c r="F17" s="3" t="n">
+        <v>9</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="7" t="inlineStr">
@@ -803,6 +849,9 @@
       <c r="E18" s="3" t="n">
         <v>10</v>
       </c>
+      <c r="F18" s="3" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="8" t="inlineStr">
@@ -849,6 +898,18 @@
       <c r="B23" s="9" t="inlineStr">
         <is>
           <t>Local: frontend :5174, API :3100; assistant model not configured (no NVIDIA_API_KEY). Browser pane already signed in to the seeded account with the readable EPUB; desktop (800px pane) and phone 375x812.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="8" t="inlineStr">
+        <is>
+          <t>Round 5 (2026-10-28)</t>
+        </is>
+      </c>
+      <c r="B24" s="9" t="inlineStr">
+        <is>
+          <t>Local: frontend :5174, API :3100 with AI_PROVIDER=nvidia and a real NVIDIA_API_KEY (live model calls, no mock). Seeded fresh account (qa.round5.1793127205@bunko.test) with AI consent pre-granted, a small library, two shelves, and one readable EPUB.</t>
         </is>
       </c>
     </row>
@@ -863,7 +924,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N79"/>
+  <dimension ref="A1:N88"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -5713,8 +5774,458 @@
       </c>
       <c r="N79" s="10" t="inlineStr"/>
     </row>
+    <row r="80">
+      <c r="A80" s="10" t="n">
+        <v>5</v>
+      </c>
+      <c r="B80" s="10" t="inlineStr">
+        <is>
+          <t>R5-01</t>
+        </is>
+      </c>
+      <c r="C80" s="10" t="inlineStr">
+        <is>
+          <t>Shelves organizing</t>
+        </is>
+      </c>
+      <c r="D80" s="10" t="inlineStr">
+        <is>
+          <t>blocker</t>
+        </is>
+      </c>
+      <c r="E80" s="10" t="inlineStr">
+        <is>
+          <t>"Add book" button in the Shelves page's "Add books to [shelf]" dialog does not work</t>
+        </is>
+      </c>
+      <c r="F80" s="10" t="inlineStr">
+        <is>
+          <t>Shelves &gt; created a new shelf 'rainy day reads' via '+ New Shelf' &gt; clicked 'Add books' on the empty shelf &gt; checked Circe and Piranesi &gt; clicked 'Add book' (repeated with ref clicks, coordinate clicks, and Enter while focused).</t>
+        </is>
+      </c>
+      <c r="G80" s="10" t="inlineStr">
+        <is>
+          <t>Selected books get added to the shelf and the dialog closes/updates the count.</t>
+        </is>
+      </c>
+      <c r="H80" s="10" t="inlineStr">
+        <is>
+          <t>Nothing happens -- dialog stays open, shelf still shows '0 books'. Workaround: toggling the shelf tag on each book's own detail page works correctly.</t>
+        </is>
+      </c>
+      <c r="I80" s="10" t="inlineStr"/>
+      <c r="J80" s="10" t="inlineStr"/>
+      <c r="K80" s="10" t="inlineStr"/>
+      <c r="L80" s="10" t="inlineStr"/>
+      <c r="M80" s="10" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="N80" s="10" t="inlineStr"/>
+    </row>
+    <row r="81">
+      <c r="A81" s="10" t="n">
+        <v>5</v>
+      </c>
+      <c r="B81" s="10" t="inlineStr">
+        <is>
+          <t>R5-02</t>
+        </is>
+      </c>
+      <c r="C81" s="10" t="inlineStr">
+        <is>
+          <t>Tracking journal statistics</t>
+        </is>
+      </c>
+      <c r="D81" s="10" t="inlineStr">
+        <is>
+          <t>major</t>
+        </is>
+      </c>
+      <c r="E81" s="10" t="inlineStr">
+        <is>
+          <t>Reflection typed into the reader's "Session ended" dialog is never saved</t>
+        </is>
+      </c>
+      <c r="F81" s="10" t="inlineStr">
+        <is>
+          <t>Finished 'The Lantern Keeper of Aldmere' in the reader &gt; 'Close the book' &gt; 'Session ended / 6 min of reading. Nice work.' dialog &gt; typed a reflection &gt; Save.</t>
+        </is>
+      </c>
+      <c r="G81" s="10" t="inlineStr">
+        <is>
+          <t>The reflection text appears in the Journal entry, the book's Notes, or its Review.</t>
+        </is>
+      </c>
+      <c r="H81" s="10" t="inlineStr">
+        <is>
+          <t>The reflection text is gone entirely. The Journal entry shows an unrelated earlier highlight instead; Notes/Review stay empty even after reload.</t>
+        </is>
+      </c>
+      <c r="I81" s="10" t="inlineStr"/>
+      <c r="J81" s="10" t="inlineStr"/>
+      <c r="K81" s="10" t="inlineStr"/>
+      <c r="L81" s="10" t="inlineStr"/>
+      <c r="M81" s="10" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="N81" s="10" t="inlineStr"/>
+    </row>
+    <row r="82">
+      <c r="A82" s="10" t="n">
+        <v>5</v>
+      </c>
+      <c r="B82" s="10" t="inlineStr">
+        <is>
+          <t>R5-03</t>
+        </is>
+      </c>
+      <c r="C82" s="10" t="inlineStr">
+        <is>
+          <t>Tracking journal statistics</t>
+        </is>
+      </c>
+      <c r="D82" s="10" t="inlineStr">
+        <is>
+          <t>minor</t>
+        </is>
+      </c>
+      <c r="E82" s="10" t="inlineStr">
+        <is>
+          <t>Logged reading session date is off by one day</t>
+        </is>
+      </c>
+      <c r="F82" s="10" t="inlineStr">
+        <is>
+          <t>Journal &gt; 'Log reading' &gt; book Piranesi, Day field showed '28-10-2026' (today), Minutes 45, From page 10, To page 55, reflection text, 'Log reading'.</t>
+        </is>
+      </c>
+      <c r="G82" s="10" t="inlineStr">
+        <is>
+          <t>Journal entry shows 'Oct 28, 2026' matching the selected date.</t>
+        </is>
+      </c>
+      <c r="H82" s="10" t="inlineStr">
+        <is>
+          <t>Entry is listed under 'Oct 27, 2026' -- one day earlier, suggesting a timezone conversion bug.</t>
+        </is>
+      </c>
+      <c r="I82" s="10" t="inlineStr"/>
+      <c r="J82" s="10" t="inlineStr"/>
+      <c r="K82" s="10" t="inlineStr"/>
+      <c r="L82" s="10" t="inlineStr"/>
+      <c r="M82" s="10" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="N82" s="10" t="inlineStr"/>
+    </row>
+    <row r="83">
+      <c r="A83" s="10" t="n">
+        <v>5</v>
+      </c>
+      <c r="B83" s="10" t="inlineStr">
+        <is>
+          <t>R5-04</t>
+        </is>
+      </c>
+      <c r="C83" s="10" t="inlineStr">
+        <is>
+          <t>Assistant chat</t>
+        </is>
+      </c>
+      <c r="D83" s="10" t="inlineStr">
+        <is>
+          <t>major</t>
+        </is>
+      </c>
+      <c r="E83" s="10" t="inlineStr">
+        <is>
+          <t>Off-topic assistant questions reliably time out (even on retry)</t>
+        </is>
+      </c>
+      <c r="F83" s="10" t="inlineStr">
+        <is>
+          <t>In Assistant chat, after several successful book-related exchanges, sent 'whats the weather like today'. Waited 30s -&gt; timeout message. Clicked 'Try again', waited another 30s.</t>
+        </is>
+      </c>
+      <c r="G83" s="10" t="inlineStr">
+        <is>
+          <t>Either a quick graceful redirect, or at least a successful retry.</t>
+        </is>
+      </c>
+      <c r="H83" s="10" t="inlineStr">
+        <is>
+          <t>Both the original attempt and the retry timed out after ~30s each with the same message. A normal on-topic question sent right after answered correctly within ~10s, so the failure seems specific to off-topic prompts.</t>
+        </is>
+      </c>
+      <c r="I83" s="10" t="inlineStr"/>
+      <c r="J83" s="10" t="inlineStr"/>
+      <c r="K83" s="10" t="inlineStr"/>
+      <c r="L83" s="10" t="inlineStr"/>
+      <c r="M83" s="10" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="N83" s="10" t="inlineStr"/>
+    </row>
+    <row r="84">
+      <c r="A84" s="10" t="n">
+        <v>5</v>
+      </c>
+      <c r="B84" s="10" t="inlineStr">
+        <is>
+          <t>R5-05</t>
+        </is>
+      </c>
+      <c r="C84" s="10" t="inlineStr">
+        <is>
+          <t>Assistant chat</t>
+        </is>
+      </c>
+      <c r="D84" s="10" t="inlineStr">
+        <is>
+          <t>minor</t>
+        </is>
+      </c>
+      <c r="E84" s="10" t="inlineStr">
+        <is>
+          <t>Natural phrasing "i started reading circe" fails to resolve the book despite Circe being in the library and just discussed</t>
+        </is>
+      </c>
+      <c r="F84" s="10" t="inlineStr">
+        <is>
+          <t>After being recommended 'Circe by Madeline Miller' in the previous message, typed 'i started reading circe'.</t>
+        </is>
+      </c>
+      <c r="G84" s="10" t="inlineStr">
+        <is>
+          <t>The assistant recognizes 'circe' as the book just discussed and marks it Reading.</t>
+        </is>
+      </c>
+      <c r="H84" s="10" t="inlineStr">
+        <is>
+          <t>"I couldn't find a book called 'reading circe'..." -- it matched the whole phrase as a title instead of parsing 'started reading' as the verb phrase. Retyping with the full title worked.</t>
+        </is>
+      </c>
+      <c r="I84" s="10" t="inlineStr"/>
+      <c r="J84" s="10" t="inlineStr"/>
+      <c r="K84" s="10" t="inlineStr"/>
+      <c r="L84" s="10" t="inlineStr"/>
+      <c r="M84" s="10" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="N84" s="10" t="inlineStr"/>
+    </row>
+    <row r="85">
+      <c r="A85" s="10" t="n">
+        <v>5</v>
+      </c>
+      <c r="B85" s="10" t="inlineStr">
+        <is>
+          <t>R5-06</t>
+        </is>
+      </c>
+      <c r="C85" s="10" t="inlineStr">
+        <is>
+          <t>Speed reliability</t>
+        </is>
+      </c>
+      <c r="D85" s="10" t="inlineStr">
+        <is>
+          <t>major</t>
+        </is>
+      </c>
+      <c r="E85" s="10" t="inlineStr">
+        <is>
+          <t>Unexpected full session logout with no warning, not reproduced on retry</t>
+        </is>
+      </c>
+      <c r="F85" s="10" t="inlineStr">
+        <is>
+          <t>On a book detail page (The Name of the Wind), clicked 'Add note', typed a note, clicked the '+ Add note' trigger button.</t>
+        </is>
+      </c>
+      <c r="G85" s="10" t="inlineStr">
+        <is>
+          <t>Note dialog opens or note saves; if a session genuinely expired, a clear message should explain why.</t>
+        </is>
+      </c>
+      <c r="H85" s="10" t="inlineStr">
+        <is>
+          <t>The app silently navigated to /login with all session state lost, no toast or explanation. Logging back in and repeating the exact steps worked fine every subsequent time.</t>
+        </is>
+      </c>
+      <c r="I85" s="10" t="inlineStr"/>
+      <c r="J85" s="10" t="inlineStr"/>
+      <c r="K85" s="10" t="inlineStr"/>
+      <c r="L85" s="10" t="inlineStr"/>
+      <c r="M85" s="10" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="N85" s="10" t="inlineStr"/>
+    </row>
+    <row r="86">
+      <c r="A86" s="10" t="n">
+        <v>5</v>
+      </c>
+      <c r="B86" s="10" t="inlineStr">
+        <is>
+          <t>R5-07</t>
+        </is>
+      </c>
+      <c r="C86" s="10" t="inlineStr">
+        <is>
+          <t>Look and feel</t>
+        </is>
+      </c>
+      <c r="D86" s="10" t="inlineStr">
+        <is>
+          <t>minor</t>
+        </is>
+      </c>
+      <c r="E86" s="10" t="inlineStr">
+        <is>
+          <t>Toolbar tooltip/panel overlays get stuck open and block clicks underneath</t>
+        </is>
+      </c>
+      <c r="F86" s="10" t="inlineStr">
+        <is>
+          <t>In the reader, clicked the Translate icon (shows 'isn't set up on this server yet' tooltip), then clicked other toolbar icons or chapter-list entries without first dismissing the Translate tooltip.</t>
+        </is>
+      </c>
+      <c r="G86" s="10" t="inlineStr">
+        <is>
+          <t>Clicking elsewhere should dismiss the previous tooltip automatically, or at least not intercept the click.</t>
+        </is>
+      </c>
+      <c r="H86" s="10" t="inlineStr">
+        <is>
+          <t>The tooltip stays on top, intercepting clicks meant for elements beneath it. Escape or its own close button dismisses it, but a casual user wouldn't know to do that and would think the buttons are broken.</t>
+        </is>
+      </c>
+      <c r="I86" s="10" t="inlineStr"/>
+      <c r="J86" s="10" t="inlineStr"/>
+      <c r="K86" s="10" t="inlineStr"/>
+      <c r="L86" s="10" t="inlineStr"/>
+      <c r="M86" s="10" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="N86" s="10" t="inlineStr"/>
+    </row>
+    <row r="87">
+      <c r="A87" s="10" t="n">
+        <v>5</v>
+      </c>
+      <c r="B87" s="10" t="inlineStr">
+        <is>
+          <t>R5-08</t>
+        </is>
+      </c>
+      <c r="C87" s="10" t="inlineStr">
+        <is>
+          <t>Library adding finding books</t>
+        </is>
+      </c>
+      <c r="D87" s="10" t="inlineStr">
+        <is>
+          <t>minor</t>
+        </is>
+      </c>
+      <c r="E87" s="10" t="inlineStr">
+        <is>
+          <t>Library grid cover art falls back to a generic placeholder even when real cover art exists</t>
+        </is>
+      </c>
+      <c r="F87" s="10" t="inlineStr">
+        <is>
+          <t>Added 'The Name of the Wind' via the Assistant, then viewed the Library grid.</t>
+        </is>
+      </c>
+      <c r="G87" s="10" t="inlineStr">
+        <is>
+          <t>Since the book's detail page and quick-view popup both show real cover art, the grid thumbnail should match.</t>
+        </is>
+      </c>
+      <c r="H87" s="10" t="inlineStr">
+        <is>
+          <t>The Library grid shows a generic orange 'T' placeholder tile, while every other metadata field is correctly enriched.</t>
+        </is>
+      </c>
+      <c r="I87" s="10" t="inlineStr"/>
+      <c r="J87" s="10" t="inlineStr"/>
+      <c r="K87" s="10" t="inlineStr"/>
+      <c r="L87" s="10" t="inlineStr"/>
+      <c r="M87" s="10" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="N87" s="10" t="inlineStr"/>
+    </row>
+    <row r="88">
+      <c r="A88" s="10" t="n">
+        <v>5</v>
+      </c>
+      <c r="B88" s="10" t="inlineStr">
+        <is>
+          <t>R5-09</t>
+        </is>
+      </c>
+      <c r="C88" s="10" t="inlineStr">
+        <is>
+          <t>Tracking journal statistics</t>
+        </is>
+      </c>
+      <c r="D88" s="10" t="inlineStr">
+        <is>
+          <t>polish</t>
+        </is>
+      </c>
+      <c r="E88" s="10" t="inlineStr">
+        <is>
+          <t>Settings page AI-features copy contradicts actual working behavior</t>
+        </is>
+      </c>
+      <c r="F88" s="10" t="inlineStr">
+        <is>
+          <t>Settings &gt; 'AI features' section.</t>
+        </is>
+      </c>
+      <c r="G88" s="10" t="inlineStr">
+        <is>
+          <t>Messaging consistent with the Assistant chat being clearly live and working with a real AI model.</t>
+        </is>
+      </c>
+      <c r="H88" s="10" t="inlineStr">
+        <is>
+          <t>Footer text reads "AI features aren't set up on this server yet -- your choice is saved for when they are", which is stale and could confuse a user about whether their data is actually being sent anywhere.</t>
+        </is>
+      </c>
+      <c r="I88" s="10" t="inlineStr"/>
+      <c r="J88" s="10" t="inlineStr"/>
+      <c r="K88" s="10" t="inlineStr"/>
+      <c r="L88" s="10" t="inlineStr"/>
+      <c r="M88" s="10" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="N88" s="10" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:N79"/>
+  <autoFilter ref="A1:N88"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -11923,4 +12434,812 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:N35"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="9" customWidth="1" min="2" max="2"/>
+    <col width="90" customWidth="1" min="3" max="3"/>
+    <col width="13" customWidth="1" min="4" max="4"/>
+    <col width="36" customWidth="1" min="5" max="5"/>
+    <col width="46" customWidth="1" min="6" max="6"/>
+    <col width="36" customWidth="1" min="7" max="7"/>
+    <col width="46" customWidth="1" min="8" max="8"/>
+    <col width="40" customWidth="1" min="9" max="9"/>
+    <col width="52" customWidth="1" min="10" max="10"/>
+    <col width="40" customWidth="1" min="11" max="11"/>
+    <col width="13" customWidth="1" min="12" max="12"/>
+    <col width="13" customWidth="1" min="13" max="13"/>
+    <col width="13" customWidth="1" min="14" max="14"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="11" t="inlineStr">
+        <is>
+          <t>Round 5</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Meera, book-lover persona (code-blind agent; browser only)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Local: frontend :5174, API :3100 with AI_PROVIDER=nvidia and a real NVIDIA_API_KEY (live model calls, no mock). Seeded fresh account (qa.round5.1793127205@bunko.test) with AI consent pre-granted, a small library, two shelves, and one readable EPUB.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>Area</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Score</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>Tester's reason</t>
+        </is>
+      </c>
+    </row>
+    <row r="5"/>
+    <row r="6">
+      <c r="A6" s="10" t="inlineStr">
+        <is>
+          <t>First impression onboarding</t>
+        </is>
+      </c>
+      <c r="B6" s="13" t="n">
+        <v>8</v>
+      </c>
+      <c r="C6" s="10" t="inlineStr">
+        <is>
+          <t>Clean, calm, book-themed login; already signed in to the seeded account so full onboarding wasn't seen, but nothing felt generic.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="10" t="inlineStr">
+        <is>
+          <t>Library adding finding books</t>
+        </is>
+      </c>
+      <c r="B7" s="12" t="n">
+        <v>7</v>
+      </c>
+      <c r="C7" s="10" t="inlineStr">
+        <is>
+          <t>Adding by title/author with real metadata/cover enrichment works well, but the library grid shows a generic placeholder tile even when the book's detail page has a real cover.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="10" t="inlineStr">
+        <is>
+          <t>Book page and details</t>
+        </is>
+      </c>
+      <c r="B8" s="13" t="n">
+        <v>8</v>
+      </c>
+      <c r="C8" s="10" t="inlineStr">
+        <is>
+          <t>Rich, well-organized page (description, series, shelves, rating, review, notes, highlights); rating and notes persisted reliably on retest.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="10" t="inlineStr">
+        <is>
+          <t>Reading experience</t>
+        </is>
+      </c>
+      <c r="B9" s="13" t="n">
+        <v>9</v>
+      </c>
+      <c r="C9" s="10" t="inlineStr">
+        <is>
+          <t>Genuinely delightful EPUB reader: 3D-flip and scroll modes, 4 legible themes, font/line/margin controls, in-book search, working highlights, bookmarks, and a thoughtful end-of-book flow.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="10" t="inlineStr">
+        <is>
+          <t>Tracking journal statistics</t>
+        </is>
+      </c>
+      <c r="B10" s="12" t="n">
+        <v>6</v>
+      </c>
+      <c r="C10" s="10" t="inlineStr">
+        <is>
+          <t>Logging/viewing/deleting sessions works with a nice delete confirmation, but a logged date was off by one day and a typed session reflection was silently discarded.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="10" t="inlineStr">
+        <is>
+          <t>Shelves organizing</t>
+        </is>
+      </c>
+      <c r="B11" s="12" t="n">
+        <v>6</v>
+      </c>
+      <c r="C11" s="10" t="inlineStr">
+        <is>
+          <t>The physical bookshelf visualization is the best-looking part of the app, but the Shelves page's own 'Add books to shelf' dialog does nothing when you click Add book.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="10" t="inlineStr">
+        <is>
+          <t>Notes highlights reviews</t>
+        </is>
+      </c>
+      <c r="B12" s="12" t="n">
+        <v>7</v>
+      </c>
+      <c r="C12" s="10" t="inlineStr">
+        <is>
+          <t>Highlighting with the color picker, the Highlights sidebar, and reviews/ratings/notes all saved and persisted, but the lost session reflection and some first-attempt save fragility hold it back.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="10" t="inlineStr">
+        <is>
+          <t>Assistant chat</t>
+        </is>
+      </c>
+      <c r="B13" s="12" t="n">
+        <v>7</v>
+      </c>
+      <c r="C13" s="10" t="inlineStr">
+        <is>
+          <t>Accurate and grounded on in-scope library questions with a working undo and clear loading states, but off-topic questions reliably time out even on retry, and 'i started reading circe' fails to parse despite Circe being the book just recommended.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="10" t="inlineStr">
+        <is>
+          <t>Look and feel</t>
+        </is>
+      </c>
+      <c r="B14" s="13" t="n">
+        <v>9</v>
+      </c>
+      <c r="C14" s="10" t="inlineStr">
+        <is>
+          <t>Serif typography, warm paper palette, the physical bookshelf, thoughtful copy, and a transparent AI-data-use settings page -- feels made by book people, not a generic template.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="10" t="inlineStr">
+        <is>
+          <t>Speed reliability</t>
+        </is>
+      </c>
+      <c r="B15" s="12" t="n">
+        <v>6</v>
+      </c>
+      <c r="C15" s="10" t="inlineStr">
+        <is>
+          <t>Most interactions are fast, but real reproducible bugs surfaced: the broken shelf add-books dialog, a lost session reflection, an off-by-one journal date, one unexplained mid-session logout, and tooltips that get stuck open and block clicks underneath.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="10" t="inlineStr">
+        <is>
+          <t>Overall</t>
+        </is>
+      </c>
+      <c r="B16" s="12" t="n">
+        <v>7</v>
+      </c>
+      <c r="C16" s="10" t="inlineStr">
+        <is>
+          <t>A charming, well-designed reading app with one of the best in-browser EPUB readers tested, let down by a handful of real functional bugs a careful reader would hit within a single normal session.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="8" t="inlineStr">
+        <is>
+          <t>Issues and fixes</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>Round</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>ID</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>Area</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>Severity</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="inlineStr">
+        <is>
+          <t>Title</t>
+        </is>
+      </c>
+      <c r="F19" s="2" t="inlineStr">
+        <is>
+          <t>Steps</t>
+        </is>
+      </c>
+      <c r="G19" s="2" t="inlineStr">
+        <is>
+          <t>Expected</t>
+        </is>
+      </c>
+      <c r="H19" s="2" t="inlineStr">
+        <is>
+          <t>Actual</t>
+        </is>
+      </c>
+      <c r="I19" s="2" t="inlineStr">
+        <is>
+          <t>Root cause</t>
+        </is>
+      </c>
+      <c r="J19" s="2" t="inlineStr">
+        <is>
+          <t>Fix</t>
+        </is>
+      </c>
+      <c r="K19" s="2" t="inlineStr">
+        <is>
+          <t>Files</t>
+        </is>
+      </c>
+      <c r="L19" s="2" t="inlineStr">
+        <is>
+          <t>Commit</t>
+        </is>
+      </c>
+      <c r="M19" s="2" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="N19" s="2" t="inlineStr">
+        <is>
+          <t>Verified in round</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="10" t="n">
+        <v>5</v>
+      </c>
+      <c r="B20" s="10" t="inlineStr">
+        <is>
+          <t>R5-01</t>
+        </is>
+      </c>
+      <c r="C20" s="10" t="inlineStr">
+        <is>
+          <t>Shelves organizing</t>
+        </is>
+      </c>
+      <c r="D20" s="10" t="inlineStr">
+        <is>
+          <t>blocker</t>
+        </is>
+      </c>
+      <c r="E20" s="10" t="inlineStr">
+        <is>
+          <t>"Add book" button in the Shelves page's "Add books to [shelf]" dialog does not work</t>
+        </is>
+      </c>
+      <c r="F20" s="10" t="inlineStr">
+        <is>
+          <t>Shelves &gt; created a new shelf 'rainy day reads' via '+ New Shelf' &gt; clicked 'Add books' on the empty shelf &gt; checked Circe and Piranesi &gt; clicked 'Add book' (repeated with ref clicks, coordinate clicks, and Enter while focused).</t>
+        </is>
+      </c>
+      <c r="G20" s="10" t="inlineStr">
+        <is>
+          <t>Selected books get added to the shelf and the dialog closes/updates the count.</t>
+        </is>
+      </c>
+      <c r="H20" s="10" t="inlineStr">
+        <is>
+          <t>Nothing happens -- dialog stays open, shelf still shows '0 books'. Workaround: toggling the shelf tag on each book's own detail page works correctly.</t>
+        </is>
+      </c>
+      <c r="I20" s="10" t="inlineStr"/>
+      <c r="J20" s="10" t="inlineStr"/>
+      <c r="K20" s="10" t="inlineStr"/>
+      <c r="L20" s="10" t="inlineStr"/>
+      <c r="M20" s="10" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="N20" s="10" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="10" t="n">
+        <v>5</v>
+      </c>
+      <c r="B21" s="10" t="inlineStr">
+        <is>
+          <t>R5-02</t>
+        </is>
+      </c>
+      <c r="C21" s="10" t="inlineStr">
+        <is>
+          <t>Tracking journal statistics</t>
+        </is>
+      </c>
+      <c r="D21" s="10" t="inlineStr">
+        <is>
+          <t>major</t>
+        </is>
+      </c>
+      <c r="E21" s="10" t="inlineStr">
+        <is>
+          <t>Reflection typed into the reader's "Session ended" dialog is never saved</t>
+        </is>
+      </c>
+      <c r="F21" s="10" t="inlineStr">
+        <is>
+          <t>Finished 'The Lantern Keeper of Aldmere' in the reader &gt; 'Close the book' &gt; 'Session ended / 6 min of reading. Nice work.' dialog &gt; typed a reflection &gt; Save.</t>
+        </is>
+      </c>
+      <c r="G21" s="10" t="inlineStr">
+        <is>
+          <t>The reflection text appears in the Journal entry, the book's Notes, or its Review.</t>
+        </is>
+      </c>
+      <c r="H21" s="10" t="inlineStr">
+        <is>
+          <t>The reflection text is gone entirely. The Journal entry shows an unrelated earlier highlight instead; Notes/Review stay empty even after reload.</t>
+        </is>
+      </c>
+      <c r="I21" s="10" t="inlineStr"/>
+      <c r="J21" s="10" t="inlineStr"/>
+      <c r="K21" s="10" t="inlineStr"/>
+      <c r="L21" s="10" t="inlineStr"/>
+      <c r="M21" s="10" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="N21" s="10" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="10" t="n">
+        <v>5</v>
+      </c>
+      <c r="B22" s="10" t="inlineStr">
+        <is>
+          <t>R5-03</t>
+        </is>
+      </c>
+      <c r="C22" s="10" t="inlineStr">
+        <is>
+          <t>Tracking journal statistics</t>
+        </is>
+      </c>
+      <c r="D22" s="10" t="inlineStr">
+        <is>
+          <t>minor</t>
+        </is>
+      </c>
+      <c r="E22" s="10" t="inlineStr">
+        <is>
+          <t>Logged reading session date is off by one day</t>
+        </is>
+      </c>
+      <c r="F22" s="10" t="inlineStr">
+        <is>
+          <t>Journal &gt; 'Log reading' &gt; book Piranesi, Day field showed '28-10-2026' (today), Minutes 45, From page 10, To page 55, reflection text, 'Log reading'.</t>
+        </is>
+      </c>
+      <c r="G22" s="10" t="inlineStr">
+        <is>
+          <t>Journal entry shows 'Oct 28, 2026' matching the selected date.</t>
+        </is>
+      </c>
+      <c r="H22" s="10" t="inlineStr">
+        <is>
+          <t>Entry is listed under 'Oct 27, 2026' -- one day earlier, suggesting a timezone conversion bug.</t>
+        </is>
+      </c>
+      <c r="I22" s="10" t="inlineStr"/>
+      <c r="J22" s="10" t="inlineStr"/>
+      <c r="K22" s="10" t="inlineStr"/>
+      <c r="L22" s="10" t="inlineStr"/>
+      <c r="M22" s="10" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="N22" s="10" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="10" t="n">
+        <v>5</v>
+      </c>
+      <c r="B23" s="10" t="inlineStr">
+        <is>
+          <t>R5-04</t>
+        </is>
+      </c>
+      <c r="C23" s="10" t="inlineStr">
+        <is>
+          <t>Assistant chat</t>
+        </is>
+      </c>
+      <c r="D23" s="10" t="inlineStr">
+        <is>
+          <t>major</t>
+        </is>
+      </c>
+      <c r="E23" s="10" t="inlineStr">
+        <is>
+          <t>Off-topic assistant questions reliably time out (even on retry)</t>
+        </is>
+      </c>
+      <c r="F23" s="10" t="inlineStr">
+        <is>
+          <t>In Assistant chat, after several successful book-related exchanges, sent 'whats the weather like today'. Waited 30s -&gt; timeout message. Clicked 'Try again', waited another 30s.</t>
+        </is>
+      </c>
+      <c r="G23" s="10" t="inlineStr">
+        <is>
+          <t>Either a quick graceful redirect, or at least a successful retry.</t>
+        </is>
+      </c>
+      <c r="H23" s="10" t="inlineStr">
+        <is>
+          <t>Both the original attempt and the retry timed out after ~30s each with the same message. A normal on-topic question sent right after answered correctly within ~10s, so the failure seems specific to off-topic prompts.</t>
+        </is>
+      </c>
+      <c r="I23" s="10" t="inlineStr"/>
+      <c r="J23" s="10" t="inlineStr"/>
+      <c r="K23" s="10" t="inlineStr"/>
+      <c r="L23" s="10" t="inlineStr"/>
+      <c r="M23" s="10" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="N23" s="10" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="10" t="n">
+        <v>5</v>
+      </c>
+      <c r="B24" s="10" t="inlineStr">
+        <is>
+          <t>R5-05</t>
+        </is>
+      </c>
+      <c r="C24" s="10" t="inlineStr">
+        <is>
+          <t>Assistant chat</t>
+        </is>
+      </c>
+      <c r="D24" s="10" t="inlineStr">
+        <is>
+          <t>minor</t>
+        </is>
+      </c>
+      <c r="E24" s="10" t="inlineStr">
+        <is>
+          <t>Natural phrasing "i started reading circe" fails to resolve the book despite Circe being in the library and just discussed</t>
+        </is>
+      </c>
+      <c r="F24" s="10" t="inlineStr">
+        <is>
+          <t>After being recommended 'Circe by Madeline Miller' in the previous message, typed 'i started reading circe'.</t>
+        </is>
+      </c>
+      <c r="G24" s="10" t="inlineStr">
+        <is>
+          <t>The assistant recognizes 'circe' as the book just discussed and marks it Reading.</t>
+        </is>
+      </c>
+      <c r="H24" s="10" t="inlineStr">
+        <is>
+          <t>"I couldn't find a book called 'reading circe'..." -- it matched the whole phrase as a title instead of parsing 'started reading' as the verb phrase. Retyping with the full title worked.</t>
+        </is>
+      </c>
+      <c r="I24" s="10" t="inlineStr"/>
+      <c r="J24" s="10" t="inlineStr"/>
+      <c r="K24" s="10" t="inlineStr"/>
+      <c r="L24" s="10" t="inlineStr"/>
+      <c r="M24" s="10" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="N24" s="10" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="10" t="n">
+        <v>5</v>
+      </c>
+      <c r="B25" s="10" t="inlineStr">
+        <is>
+          <t>R5-06</t>
+        </is>
+      </c>
+      <c r="C25" s="10" t="inlineStr">
+        <is>
+          <t>Speed reliability</t>
+        </is>
+      </c>
+      <c r="D25" s="10" t="inlineStr">
+        <is>
+          <t>major</t>
+        </is>
+      </c>
+      <c r="E25" s="10" t="inlineStr">
+        <is>
+          <t>Unexpected full session logout with no warning, not reproduced on retry</t>
+        </is>
+      </c>
+      <c r="F25" s="10" t="inlineStr">
+        <is>
+          <t>On a book detail page (The Name of the Wind), clicked 'Add note', typed a note, clicked the '+ Add note' trigger button.</t>
+        </is>
+      </c>
+      <c r="G25" s="10" t="inlineStr">
+        <is>
+          <t>Note dialog opens or note saves; if a session genuinely expired, a clear message should explain why.</t>
+        </is>
+      </c>
+      <c r="H25" s="10" t="inlineStr">
+        <is>
+          <t>The app silently navigated to /login with all session state lost, no toast or explanation. Logging back in and repeating the exact steps worked fine every subsequent time.</t>
+        </is>
+      </c>
+      <c r="I25" s="10" t="inlineStr"/>
+      <c r="J25" s="10" t="inlineStr"/>
+      <c r="K25" s="10" t="inlineStr"/>
+      <c r="L25" s="10" t="inlineStr"/>
+      <c r="M25" s="10" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="N25" s="10" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="10" t="n">
+        <v>5</v>
+      </c>
+      <c r="B26" s="10" t="inlineStr">
+        <is>
+          <t>R5-07</t>
+        </is>
+      </c>
+      <c r="C26" s="10" t="inlineStr">
+        <is>
+          <t>Look and feel</t>
+        </is>
+      </c>
+      <c r="D26" s="10" t="inlineStr">
+        <is>
+          <t>minor</t>
+        </is>
+      </c>
+      <c r="E26" s="10" t="inlineStr">
+        <is>
+          <t>Toolbar tooltip/panel overlays get stuck open and block clicks underneath</t>
+        </is>
+      </c>
+      <c r="F26" s="10" t="inlineStr">
+        <is>
+          <t>In the reader, clicked the Translate icon (shows 'isn't set up on this server yet' tooltip), then clicked other toolbar icons or chapter-list entries without first dismissing the Translate tooltip.</t>
+        </is>
+      </c>
+      <c r="G26" s="10" t="inlineStr">
+        <is>
+          <t>Clicking elsewhere should dismiss the previous tooltip automatically, or at least not intercept the click.</t>
+        </is>
+      </c>
+      <c r="H26" s="10" t="inlineStr">
+        <is>
+          <t>The tooltip stays on top, intercepting clicks meant for elements beneath it. Escape or its own close button dismisses it, but a casual user wouldn't know to do that and would think the buttons are broken.</t>
+        </is>
+      </c>
+      <c r="I26" s="10" t="inlineStr"/>
+      <c r="J26" s="10" t="inlineStr"/>
+      <c r="K26" s="10" t="inlineStr"/>
+      <c r="L26" s="10" t="inlineStr"/>
+      <c r="M26" s="10" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="N26" s="10" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="10" t="n">
+        <v>5</v>
+      </c>
+      <c r="B27" s="10" t="inlineStr">
+        <is>
+          <t>R5-08</t>
+        </is>
+      </c>
+      <c r="C27" s="10" t="inlineStr">
+        <is>
+          <t>Library adding finding books</t>
+        </is>
+      </c>
+      <c r="D27" s="10" t="inlineStr">
+        <is>
+          <t>minor</t>
+        </is>
+      </c>
+      <c r="E27" s="10" t="inlineStr">
+        <is>
+          <t>Library grid cover art falls back to a generic placeholder even when real cover art exists</t>
+        </is>
+      </c>
+      <c r="F27" s="10" t="inlineStr">
+        <is>
+          <t>Added 'The Name of the Wind' via the Assistant, then viewed the Library grid.</t>
+        </is>
+      </c>
+      <c r="G27" s="10" t="inlineStr">
+        <is>
+          <t>Since the book's detail page and quick-view popup both show real cover art, the grid thumbnail should match.</t>
+        </is>
+      </c>
+      <c r="H27" s="10" t="inlineStr">
+        <is>
+          <t>The Library grid shows a generic orange 'T' placeholder tile, while every other metadata field is correctly enriched.</t>
+        </is>
+      </c>
+      <c r="I27" s="10" t="inlineStr"/>
+      <c r="J27" s="10" t="inlineStr"/>
+      <c r="K27" s="10" t="inlineStr"/>
+      <c r="L27" s="10" t="inlineStr"/>
+      <c r="M27" s="10" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="N27" s="10" t="inlineStr"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="10" t="n">
+        <v>5</v>
+      </c>
+      <c r="B28" s="10" t="inlineStr">
+        <is>
+          <t>R5-09</t>
+        </is>
+      </c>
+      <c r="C28" s="10" t="inlineStr">
+        <is>
+          <t>Tracking journal statistics</t>
+        </is>
+      </c>
+      <c r="D28" s="10" t="inlineStr">
+        <is>
+          <t>polish</t>
+        </is>
+      </c>
+      <c r="E28" s="10" t="inlineStr">
+        <is>
+          <t>Settings page AI-features copy contradicts actual working behavior</t>
+        </is>
+      </c>
+      <c r="F28" s="10" t="inlineStr">
+        <is>
+          <t>Settings &gt; 'AI features' section.</t>
+        </is>
+      </c>
+      <c r="G28" s="10" t="inlineStr">
+        <is>
+          <t>Messaging consistent with the Assistant chat being clearly live and working with a real AI model.</t>
+        </is>
+      </c>
+      <c r="H28" s="10" t="inlineStr">
+        <is>
+          <t>Footer text reads "AI features aren't set up on this server yet -- your choice is saved for when they are", which is stale and could confuse a user about whether their data is actually being sent anywhere.</t>
+        </is>
+      </c>
+      <c r="I28" s="10" t="inlineStr"/>
+      <c r="J28" s="10" t="inlineStr"/>
+      <c r="K28" s="10" t="inlineStr"/>
+      <c r="L28" s="10" t="inlineStr"/>
+      <c r="M28" s="10" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="N28" s="10" t="inlineStr"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="8" t="inlineStr">
+        <is>
+          <t>What the tester liked</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>The 3D-flip/scroll EPUB reader is excellent: real pagination with chapter titles, 4 legible reading themes, font/line-spacing/margin controls, in-book search that jumps to the exact page, and highlights that persist across reload.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>The physical bookshelf visualization on the Shelves page (wood shelf texture, genre grouping, Covers/Spines toggle, drag to rearrange) is delightful and unlike any generic tracker UI.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>The Assistant correctly grounds its answers in the user's actual library (accurate counts, correct want-to-read list, sensible recommendations) and has a working, reliable undo for its last action.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>The 'Session ended' flow after finishing a book (reading-time summary, 'Finished [Book]?' prompt, auto-set finish date) mirrors how a real reader thinks about wrapping up a book.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>Settings' AI-features section is unusually transparent about exactly what data is sent to which third-party service and when -- genuinely trust-building rather than generic boilerplate.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>